<commit_message>
se actualziaron los flujos
</commit_message>
<xml_diff>
--- a/docs/assets/infraestructura/s1-e1-matriz-componentes-red.xlsx
+++ b/docs/assets/infraestructura/s1-e1-matriz-componentes-red.xlsx
@@ -516,7 +516,7 @@
     <col min="4" max="4" width="11.83203125" customWidth="1"/>
     <col min="5" max="5" width="60.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="46.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
     <col min="8" max="8" width="37.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -878,7 +878,7 @@
         <v>Alta</v>
       </c>
       <c r="G14" t="str">
-        <v>Diseñado (hoy en la PC local)</v>
+        <v>Diseñado (hoy en el VPS)</v>
       </c>
       <c r="H14" t="str">
         <v>General, Lógica, Zonas, Hipervisor</v>
@@ -1132,7 +1132,7 @@
         <v>NUBE</v>
       </c>
       <c r="E24" t="str">
-        <v>Sistema del colegio, extremo VPN y proxy inverso</v>
+        <v>Sistema del colegio, capa relacional de la academia (desde el 2026-10-24), extremo VPN y proxy inverso</v>
       </c>
       <c r="F24" t="str">
         <v>Crítica</v>
@@ -1184,7 +1184,7 @@
         <v>NUBE</v>
       </c>
       <c r="E26" t="str">
-        <v>Servidor web, API del colegio y proxy inverso hacia la sede</v>
+        <v>Servidor web, API del colegio, sitios api-academia y analitica-academia, y proxy inverso hacia la sede</v>
       </c>
       <c r="F26" t="str">
         <v>Crítica</v>
@@ -1331,7 +1331,7 @@
         <v>NET-31</v>
       </c>
       <c r="B32" t="str">
-        <v>PC local actual (API, MySQL y analítica con PM2)</v>
+        <v>PC local (antes: API, MySQL y analítica con PM2)</v>
       </c>
       <c r="C32" t="str">
         <v>Red actual de la sede, sin segmentar</v>
@@ -1340,13 +1340,13 @@
         <v>Actual</v>
       </c>
       <c r="E32" t="str">
-        <v>Réplica relacional y analítica hasta migrar a VM-APP01</v>
+        <v>Entorno anterior de la réplica; desde el 2026-10-24 solo pruebas de restauración</v>
       </c>
       <c r="F32" t="str">
         <v>Media</v>
       </c>
       <c r="G32" t="str">
-        <v>Implementado (transitorio)</v>
+        <v>Retirado (2026-10-24): la capa corre en el VPS</v>
       </c>
       <c r="H32" t="str">
         <v>General</v>
@@ -3093,11 +3093,11 @@
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="51.83203125" customWidth="1"/>
-    <col min="3" max="3" width="51.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
     <col min="4" max="4" width="42.83203125" customWidth="1"/>
     <col min="5" max="5" width="58.83203125" customWidth="1"/>
     <col min="6" max="6" width="28.83203125" customWidth="1"/>
-    <col min="7" max="7" width="54.83203125" customWidth="1"/>
+    <col min="7" max="7" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3177,7 +3177,7 @@
         <v>Navegador (admin, docente, auxiliar)</v>
       </c>
       <c r="C4" t="str">
-        <v>Proxy del VPS (subdominio propuesto api-academia)</v>
+        <v>Nginx del VPS (api-academia.cermatschool.edu.pe)</v>
       </c>
       <c r="D4" t="str">
         <v>HTTPS 443/tcp</v>
@@ -3189,7 +3189,7 @@
         <v>Internet</v>
       </c>
       <c r="G4" t="str">
-        <v>Pendiente (hoy http://localhost:3001 en la PC local)</v>
+        <v>Implementado (2026-10-24); prueba de punta a punta con respuesta 200</v>
       </c>
     </row>
     <row r="5">
@@ -3212,7 +3212,7 @@
         <v>Túnel IPsec</v>
       </c>
       <c r="G5" t="str">
-        <v>Pendiente</v>
+        <v>Pendiente (hoy Nginx entrega a la API y la analítica en 127.0.0.1 del mismo VPS)</v>
       </c>
     </row>
     <row r="6">
@@ -3235,7 +3235,7 @@
         <v>Internet (NAT de OPNsense)</v>
       </c>
       <c r="G6" t="str">
-        <v>Implementado en la PC local</v>
+        <v>Implementado en el VPS (2026-10-24)</v>
       </c>
     </row>
     <row r="7">
@@ -3258,7 +3258,7 @@
         <v>Local</v>
       </c>
       <c r="G7" t="str">
-        <v>Implementado en la PC local</v>
+        <v>Implementado en el VPS (2026-10-24)</v>
       </c>
     </row>
     <row r="8">

</xml_diff>